<commit_message>
Extend DCF projections to 10 years and update related calculations
Co-authored-by: luizeduardop <luizeduardop@gmail.com>
</commit_message>
<xml_diff>
--- a/Mining_Contractor_Valuation_Model.xlsx
+++ b/Mining_Contractor_Valuation_Model.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Financial Data Input" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Historical Analysis" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DCF Valuation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Comparable Analysis" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Precedent Transactions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Asset-Based Valuation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Valuation Summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sensitivity Analysis" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Risk Analysis" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Data Input" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Analysis" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF Valuation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparable Analysis" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precedent Transactions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset-Based Valuation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation Summary" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity Analysis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Analysis" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2401,40 +2401,50 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EBITDA Margin (Terminal)</t>
+          <t>Revenue Growth Rate (Years 6-10)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Capex as % of Revenue</t>
+          <t>EBITDA Margin (Terminal)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Working Capital as % of Revenue</t>
+          <t>Capex as % of Revenue</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Working Capital as % of Revenue</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Depreciation as % of Capex</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>80</v>
       </c>
     </row>
@@ -2703,40 +2713,240 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>2030</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2031</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2032</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2033</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2034</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2755,7 +2965,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sum of PV of FCF (2025-2029)</t>
+          <t>Sum of PV of FCF (2025-2034)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -3916,7 +4126,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Based on 5-year projections</t>
+          <t>Based on 10-year projections</t>
         </is>
       </c>
     </row>

</xml_diff>